<commit_message>
Add demographic distribution analytics
</commit_message>
<xml_diff>
--- a/kit-free/datos-ejemplo/plantilla-demografica-ejemplo.xlsx
+++ b/kit-free/datos-ejemplo/plantilla-demografica-ejemplo.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:S41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -446,6 +446,18 @@
       <c r="O1" t="str">
         <v>NivelPuesto</v>
       </c>
+      <c r="P1" t="str">
+        <v>Provincia</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Nacionalidad</v>
+      </c>
+      <c r="R1" t="str">
+        <v>FechaInicioPuesto</v>
+      </c>
+      <c r="S1" t="str">
+        <v>JornadaSemanal</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -493,6 +505,18 @@
       <c r="O2" t="str">
         <v>Junior</v>
       </c>
+      <c r="P2" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R2" t="str">
+        <v>2023-01-09</v>
+      </c>
+      <c r="S2" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -540,6 +564,18 @@
       <c r="O3" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P3" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R3" t="str">
+        <v>2023-01-16</v>
+      </c>
+      <c r="S3" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -587,6 +623,18 @@
       <c r="O4" t="str">
         <v>Senior</v>
       </c>
+      <c r="P4" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R4" t="str">
+        <v>2023-02-06</v>
+      </c>
+      <c r="S4" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -634,6 +682,18 @@
       <c r="O5" t="str">
         <v>Manager</v>
       </c>
+      <c r="P5" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R5" t="str">
+        <v>2023-02-20</v>
+      </c>
+      <c r="S5" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -681,6 +741,18 @@
       <c r="O6" t="str">
         <v>Junior</v>
       </c>
+      <c r="P6" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R6" t="str">
+        <v>2023-03-13</v>
+      </c>
+      <c r="S6" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -728,6 +800,18 @@
       <c r="O7" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P7" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R7" t="str">
+        <v>2023-04-03</v>
+      </c>
+      <c r="S7" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -775,6 +859,18 @@
       <c r="O8" t="str">
         <v>Senior</v>
       </c>
+      <c r="P8" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R8" t="str">
+        <v>2023-04-17</v>
+      </c>
+      <c r="S8" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -822,6 +918,18 @@
       <c r="O9" t="str">
         <v>Manager</v>
       </c>
+      <c r="P9" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R9" t="str">
+        <v>2023-05-08</v>
+      </c>
+      <c r="S9" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -869,6 +977,18 @@
       <c r="O10" t="str">
         <v>Junior</v>
       </c>
+      <c r="P10" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R10" t="str">
+        <v>2023-06-05</v>
+      </c>
+      <c r="S10" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -916,6 +1036,18 @@
       <c r="O11" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P11" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R11" t="str">
+        <v>2023-07-03</v>
+      </c>
+      <c r="S11" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -963,6 +1095,18 @@
       <c r="O12" t="str">
         <v>Senior</v>
       </c>
+      <c r="P12" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R12" t="str">
+        <v>2023-08-14</v>
+      </c>
+      <c r="S12" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1010,6 +1154,18 @@
       <c r="O13" t="str">
         <v>Manager</v>
       </c>
+      <c r="P13" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R13" t="str">
+        <v>2023-09-04</v>
+      </c>
+      <c r="S13" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1057,6 +1213,18 @@
       <c r="O14" t="str">
         <v>Junior</v>
       </c>
+      <c r="P14" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R14" t="str">
+        <v>2023-10-02</v>
+      </c>
+      <c r="S14" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1104,6 +1272,18 @@
       <c r="O15" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P15" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R15" t="str">
+        <v>2023-11-06</v>
+      </c>
+      <c r="S15" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1151,6 +1331,18 @@
       <c r="O16" t="str">
         <v>Senior</v>
       </c>
+      <c r="P16" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R16" t="str">
+        <v>2023-12-11</v>
+      </c>
+      <c r="S16" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1198,6 +1390,18 @@
       <c r="O17" t="str">
         <v>Manager</v>
       </c>
+      <c r="P17" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R17" t="str">
+        <v>2024-01-08</v>
+      </c>
+      <c r="S17" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1245,6 +1449,18 @@
       <c r="O18" t="str">
         <v>Junior</v>
       </c>
+      <c r="P18" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R18" t="str">
+        <v>2024-01-22</v>
+      </c>
+      <c r="S18" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1292,6 +1508,18 @@
       <c r="O19" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P19" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R19" t="str">
+        <v>2024-02-05</v>
+      </c>
+      <c r="S19" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1339,6 +1567,18 @@
       <c r="O20" t="str">
         <v>Senior</v>
       </c>
+      <c r="P20" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R20" t="str">
+        <v>2024-02-19</v>
+      </c>
+      <c r="S20" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1386,6 +1626,18 @@
       <c r="O21" t="str">
         <v>Manager</v>
       </c>
+      <c r="P21" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R21" t="str">
+        <v>2024-03-04</v>
+      </c>
+      <c r="S21" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1433,6 +1685,18 @@
       <c r="O22" t="str">
         <v>Junior</v>
       </c>
+      <c r="P22" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R22" t="str">
+        <v>2024-03-18</v>
+      </c>
+      <c r="S22" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1480,6 +1744,18 @@
       <c r="O23" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P23" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R23" t="str">
+        <v>2024-04-08</v>
+      </c>
+      <c r="S23" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1527,6 +1803,18 @@
       <c r="O24" t="str">
         <v>Senior</v>
       </c>
+      <c r="P24" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R24" t="str">
+        <v>2024-05-06</v>
+      </c>
+      <c r="S24" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1574,6 +1862,18 @@
       <c r="O25" t="str">
         <v>Manager</v>
       </c>
+      <c r="P25" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R25" t="str">
+        <v>2024-06-03</v>
+      </c>
+      <c r="S25" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1621,6 +1921,18 @@
       <c r="O26" t="str">
         <v>Junior</v>
       </c>
+      <c r="P26" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R26" t="str">
+        <v>2024-07-01</v>
+      </c>
+      <c r="S26" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1668,6 +1980,18 @@
       <c r="O27" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P27" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R27" t="str">
+        <v>2024-08-05</v>
+      </c>
+      <c r="S27" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1715,6 +2039,18 @@
       <c r="O28" t="str">
         <v>Senior</v>
       </c>
+      <c r="P28" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R28" t="str">
+        <v>2024-09-02</v>
+      </c>
+      <c r="S28" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1762,6 +2098,18 @@
       <c r="O29" t="str">
         <v>Manager</v>
       </c>
+      <c r="P29" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R29" t="str">
+        <v>2024-10-07</v>
+      </c>
+      <c r="S29" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1809,6 +2157,18 @@
       <c r="O30" t="str">
         <v>Junior</v>
       </c>
+      <c r="P30" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R30" t="str">
+        <v>2024-11-04</v>
+      </c>
+      <c r="S30" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1856,6 +2216,18 @@
       <c r="O31" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P31" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R31" t="str">
+        <v>2024-12-02</v>
+      </c>
+      <c r="S31" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1903,6 +2275,18 @@
       <c r="O32" t="str">
         <v>Senior</v>
       </c>
+      <c r="P32" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R32" t="str">
+        <v>2025-01-07</v>
+      </c>
+      <c r="S32" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1950,6 +2334,18 @@
       <c r="O33" t="str">
         <v>Manager</v>
       </c>
+      <c r="P33" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R33" t="str">
+        <v>2025-01-20</v>
+      </c>
+      <c r="S33" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1997,6 +2393,18 @@
       <c r="O34" t="str">
         <v>Junior</v>
       </c>
+      <c r="P34" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R34" t="str">
+        <v>2025-02-03</v>
+      </c>
+      <c r="S34" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2044,6 +2452,18 @@
       <c r="O35" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P35" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R35" t="str">
+        <v>2025-02-17</v>
+      </c>
+      <c r="S35" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2091,6 +2511,18 @@
       <c r="O36" t="str">
         <v>Senior</v>
       </c>
+      <c r="P36" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R36" t="str">
+        <v>2025-03-03</v>
+      </c>
+      <c r="S36" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2138,6 +2570,18 @@
       <c r="O37" t="str">
         <v>Manager</v>
       </c>
+      <c r="P37" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R37" t="str">
+        <v>2025-03-17</v>
+      </c>
+      <c r="S37" t="str">
+        <v>30</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2185,6 +2629,18 @@
       <c r="O38" t="str">
         <v>Junior</v>
       </c>
+      <c r="P38" t="str">
+        <v>Barcelona</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R38" t="str">
+        <v>2025-04-01</v>
+      </c>
+      <c r="S38" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2232,6 +2688,18 @@
       <c r="O39" t="str">
         <v>Profesional</v>
       </c>
+      <c r="P39" t="str">
+        <v>Madrid</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>Española</v>
+      </c>
+      <c r="R39" t="str">
+        <v>2025-04-14</v>
+      </c>
+      <c r="S39" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2279,6 +2747,18 @@
       <c r="O40" t="str">
         <v>Senior</v>
       </c>
+      <c r="P40" t="str">
+        <v>Valencia</v>
+      </c>
+      <c r="Q40" t="str">
+        <v>Portuguesa</v>
+      </c>
+      <c r="R40" t="str">
+        <v>2025-05-05</v>
+      </c>
+      <c r="S40" t="str">
+        <v>40</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2326,10 +2806,22 @@
       <c r="O41" t="str">
         <v>Manager</v>
       </c>
+      <c r="P41" t="str">
+        <v>Sevilla</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>Italiana</v>
+      </c>
+      <c r="R41" t="str">
+        <v>2025-06-02</v>
+      </c>
+      <c r="S41" t="str">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S41"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>